<commit_message>
refactor: constantes centralizadas, filtros independientes, validación horario y fix % asistencia
- src/lib/constants.ts: fuente única para DAYS, DAY_KEYS, STATUS_LABEL/COLOR/BG, ATTENDANCE_STATUSES
- Fix bug DAY_KEYS: orden correcto para Date.getDay() (domingo=0), corrige grupos del día en dashboard
- alumnos-view: filtros "sin grupo" y búsqueda ahora son independientes y combinables
- grupos-view: validación time_end > time_start en crear y editar grupo
- generate-attendance-excel: % Asistencia cuenta "tarde" como asistido + nueva columna % Puntualidad
- Eliminadas constantes duplicadas de asistencia-view, director-asistencia-view, grupos-view, pages

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/plantillas/informe-asistencia.xlsx
+++ b/public/plantillas/informe-asistencia.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\valen\Documents\Claude\AcademyOS_v2\public\plantillas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A84AC34-65B4-431D-954F-6F90B62F8D2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FF2AFA2-6798-4B76-99B5-316610393AF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-15000" yWindow="-16425" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-15000" yWindow="-16425" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Inicio" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="7">
   <si>
     <t>Grupo</t>
   </si>
@@ -56,6 +56,9 @@
   </si>
   <si>
     <t>Resumen total de asistencia</t>
+  </si>
+  <si>
+    <t>% Puntualidad</t>
   </si>
 </sst>
 </file>
@@ -533,15 +536,15 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A11:E18"/>
+  <dimension ref="A11:F18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="4" max="4" width="17.19921875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="17.19921875" customWidth="1"/>
-    <col min="6" max="6" width="13.3984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="11" spans="1:5" ht="21" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:6" ht="21" x14ac:dyDescent="0.4">
       <c r="A11" s="5" t="s">
         <v>4</v>
       </c>
@@ -550,26 +553,29 @@
       <c r="D11" s="5"/>
       <c r="E11" s="5"/>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="D14" s="2" t="s">
         <v>3</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F14" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="D15" s="3"/>
       <c r="E15" s="3"/>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="D16" s="3"/>
       <c r="E16" s="3"/>
     </row>

</xml_diff>